<commit_message>
fixing the strict check for excel start date and end date
</commit_message>
<xml_diff>
--- a/data/menu.xlsx
+++ b/data/menu.xlsx
@@ -584,9 +584,12 @@
       <c r="B18" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="B9 B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid date format" error="Please enter date as DD/MM/YYYY (e.g., 01/03/2026)." promptTitle="Date format" prompt="Enter date in DD/MM/YYYY format." type="custom">
-      <formula1>=OR(B2="",AND(LEN(B2)=10, MID(B2,3,1)="/", MID(B2,6,1)="/"))</formula1>
+  <dataValidations count="2">
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid date format" error="Please enter date as DD/MM/YYYY (e.g., 01/03/2026)." promptTitle="Date format" prompt="Enter date in DD/MM/YYYY format." type="custom">
+      <formula1>=OR(B9="",ISNUMBER(B9),AND(LEN(B9)=10, MID(B9,3,1)="/", MID(B9,6,1)="/"))</formula1>
+    </dataValidation>
+    <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid date format" error="Please enter date as DD/MM/YYYY (e.g., 01/03/2026)." promptTitle="Date format" prompt="Enter date in DD/MM/YYYY format." type="custom">
+      <formula1>=OR(B10="",ISNUMBER(B10),AND(LEN(B10)=10, MID(B10,3,1)="/", MID(B10,6,1)="/"))</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>